<commit_message>
updated endpoints and required fields
</commit_message>
<xml_diff>
--- a/endpoints.xlsx
+++ b/endpoints.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26409"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="11" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A138466-F68F-4A72-B993-906B698E0BC3}"/>
+  <xr:revisionPtr revIDLastSave="224" documentId="11_E60897F41BE170836B02CE998F75CCDC64E183C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFAF334A-3200-42F0-AFEC-D8D5F01424EE}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="73">
+  <si>
+    <t>Prefix</t>
+  </si>
   <si>
     <t>Endpoint</t>
   </si>
@@ -39,26 +42,231 @@
     <t>Type</t>
   </si>
   <si>
-    <t>Router File</t>
+    <t>Parameters</t>
+  </si>
+  <si>
+    <t>Auth</t>
+  </si>
+  <si>
+    <t>Body requirements (optional)</t>
+  </si>
+  <si>
+    <t>events</t>
+  </si>
+  <si>
+    <t>getEvents</t>
+  </si>
+  <si>
+    <t>Gets all events in the database</t>
   </si>
   <si>
     <t>GET</t>
   </si>
   <si>
-    <t>events</t>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>getPublicEvents</t>
+  </si>
+  <si>
+    <t>Gets all events with public data only sorted by date of creation in descendent order</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>getEventById/:id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gets an event by its id (12 byte Object ID) </t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>createEvent</t>
+  </si>
+  <si>
+    <t>Creates an event</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>description, state, datetime, memberLimit, members, organizer, (chef), (shoppingDesignee)</t>
+  </si>
+  <si>
+    <t>editEvent/:id</t>
+  </si>
+  <si>
+    <t>Edits an event by its id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>PUT</t>
+  </si>
+  <si>
+    <t>Yes and user token needs to be the organizer's</t>
+  </si>
+  <si>
+    <t>description, state, datetime, memberLimit, [members], chef, shoppingDesignee, [transferReceipts], [purchaseReceipts]</t>
+  </si>
+  <si>
+    <t>deleteEvent/:id</t>
+  </si>
+  <si>
+    <t>Deletes an event by its id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>DELETE</t>
+  </si>
+  <si>
+    <t>login</t>
+  </si>
+  <si>
+    <t>Logs a user into the app</t>
+  </si>
+  <si>
+    <t>email, password</t>
+  </si>
+  <si>
+    <t>purchaseReceipt</t>
+  </si>
+  <si>
+    <t>getPurchaseReceiptsByEvent/:event</t>
+  </si>
+  <si>
+    <t>Gets all purchaseReceipts from an event providing the event's id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>event</t>
+  </si>
+  <si>
+    <t>getPurchaseReceiptById/:event</t>
+  </si>
+  <si>
+    <t>Gets a single purchaseReceipts by its id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>createPurchaseReceipt/:event</t>
+  </si>
+  <si>
+    <t>Creates a purchaseReceipt for a certain event</t>
+  </si>
+  <si>
+    <t>Yes and user token needs to be the shoppingDesignee's</t>
+  </si>
+  <si>
+    <t>description, amount, (image)</t>
+  </si>
+  <si>
+    <t>deletePurchaseReceipt/:id/:event</t>
+  </si>
+  <si>
+    <t>Deletes a purchaseReceipt by id for a certain event providig the event's id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>id, event</t>
+  </si>
+  <si>
+    <t>recoverPassword</t>
+  </si>
+  <si>
+    <t>forgot</t>
+  </si>
+  <si>
+    <t>Updates verification code for password recovery and sends the recovery email</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>recover</t>
+  </si>
+  <si>
+    <t>Changes user's password providing the correct verification code</t>
+  </si>
+  <si>
+    <t>email, verificationCode, password</t>
+  </si>
+  <si>
+    <t>transferReceipt</t>
+  </si>
+  <si>
+    <t>getTransferReceiptsByEvent/:event</t>
+  </si>
+  <si>
+    <t>Gets all transferReceipts from an event providing the event's id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>getTransferReceiptsById/:id</t>
+  </si>
+  <si>
+    <t>Gets a single transferReceipts by its id (12 byte Object ID)</t>
+  </si>
+  <si>
+    <t>createTransferPurchase/:event</t>
+  </si>
+  <si>
+    <t>Creates a transferReceipt for a certain event</t>
+  </si>
+  <si>
+    <t>description, amount, user, (paymentMethod), (image) | DON'T SEND hasPaid or send it as false</t>
+  </si>
+  <si>
+    <t>users</t>
+  </si>
+  <si>
+    <t>getUsers</t>
+  </si>
+  <si>
+    <t>Gets all users in the database</t>
+  </si>
+  <si>
+    <t>getUserById</t>
+  </si>
+  <si>
+    <t>register</t>
+  </si>
+  <si>
+    <t>Creates a user</t>
+  </si>
+  <si>
+    <t>name, email, password, profilePicture, [specialDiet], (cbu), (alias)</t>
+  </si>
+  <si>
+    <t>editUser</t>
+  </si>
+  <si>
+    <t>Edits a user by its id (12 byte Object ID) | NOT PROGRAMMED YET</t>
+  </si>
+  <si>
+    <t>deleteUser</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deletes a user by id (12 byte Object ID) | NEED TO FIX AUTH </t>
+  </si>
+  <si>
+    <t>Yes (and user token needs to be the user to delete -&gt; not functional yet)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF444444"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -69,7 +277,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -77,12 +285,77 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,33 +670,453 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="84.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="107.28515625" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="C2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>29</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" t="s">
+        <v>24</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" t="s">
+        <v>20</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D22" t="s">
+        <v>29</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>